<commit_message>
fix: use array syntax for addRow, shorten sheet names, limit validation rows
- addRow([...]) instead of addRow({...}) for Vercel compatibility
- Sheet names <31 chars: '2. Properti (Kamar, Villa)', '3. Layanan (Supir, Asuransi)'
- Validation rows: 200 -> 50 for performance
- maxDuration: 30s
</commit_message>
<xml_diff>
--- a/test_prod_v2.xlsx
+++ b/test_prod_v2.xlsx
@@ -5,8 +5,8 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="1. Armada (Kendaraan, Travel)" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="2. Properti (Kamar, Villa, Kost" state="visible" r:id="rId5"/>
-    <sheet sheetId="3" name="3. Layanan (Supir, Asuransi, Be" state="visible" r:id="rId6"/>
+    <sheet sheetId="2" name="2. Properti (Kamar, Villa, Hote" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="3. Layanan (Supir, Asuransi, Bs" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>

</xml_diff>